<commit_message>
Major cardiovascular surgery (final)
</commit_message>
<xml_diff>
--- a/codelists/major_cardiovascular_surgery_raw.xlsx
+++ b/codelists/major_cardiovascular_surgery_raw.xlsx
@@ -5928,7 +5928,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>272113010</t>
+          <t>272106010</t>
         </is>
       </c>
       <c r="B136" s="1" t="n">
@@ -5936,12 +5936,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>7A543</t>
+          <t>7A54</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>7A54300</t>
+          <t>7A54.00</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5956,20 +5956,20 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Percutaneous transluminal cannulation of artery NEC</t>
+          <t>Therapeutic transluminal operations on other artery</t>
         </is>
       </c>
       <c r="H136" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I136" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>394341010</t>
+          <t>272113010</t>
         </is>
       </c>
       <c r="B137" s="1" t="n">
@@ -5977,12 +5977,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>7A4A</t>
+          <t>7A543</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>7A4A.00</t>
+          <t>7A54300</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -5997,20 +5997,20 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Other open operations on femoral artery or popliteal artery</t>
+          <t>Percutaneous transluminal cannulation of artery NEC</t>
         </is>
       </c>
       <c r="H137" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I137" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>272106010</t>
+          <t>394341010</t>
         </is>
       </c>
       <c r="B138" s="1" t="n">
@@ -6018,12 +6018,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>7A54</t>
+          <t>7A4A</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>7A54.00</t>
+          <t>7A4A.00</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -6038,7 +6038,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Therapeutic transluminal operations on other artery</t>
+          <t>Other open operations on femoral artery or popliteal artery</t>
         </is>
       </c>
       <c r="H138" s="1" t="n">
@@ -6859,7 +6859,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>272130012</t>
+          <t>272104013</t>
         </is>
       </c>
       <c r="B159" s="1" t="n">
@@ -6867,12 +6867,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>7A5z</t>
+          <t>7A53y</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>7A5z.00</t>
+          <t>7A53y00</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -6887,7 +6887,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Other artery operations NOS</t>
+          <t>Other specified other open operation on other artery</t>
         </is>
       </c>
       <c r="H159" s="1" t="n">
@@ -6900,7 +6900,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>410979014</t>
+          <t>272130012</t>
         </is>
       </c>
       <c r="B160" s="1" t="n">
@@ -6908,12 +6908,12 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>7A4A-3</t>
+          <t>7A5z</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>7A4A.13</t>
+          <t>7A5z.00</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Other open operations on popliteal artery</t>
+          <t>Other artery operations NOS</t>
         </is>
       </c>
       <c r="H160" s="1" t="n">
@@ -6941,7 +6941,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>619411000006116</t>
+          <t>24571000006113</t>
         </is>
       </c>
       <c r="B161" s="1" t="n">
@@ -6949,12 +6949,12 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>7A55y</t>
+          <t>7A4Ay</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>7A55y00</t>
+          <t>7A4Ay00</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -6969,7 +6969,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Diagnostic transluminal operation on other artery OS</t>
+          <t>Other open operation on femoral or popliteal artery OS</t>
         </is>
       </c>
       <c r="H161" s="1" t="n">
@@ -6982,7 +6982,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>24571000006113</t>
+          <t>619411000006116</t>
         </is>
       </c>
       <c r="B162" s="1" t="n">
@@ -6990,12 +6990,12 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>7A4Ay</t>
+          <t>7A55y</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>7A4Ay00</t>
+          <t>7A55y00</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
@@ -7010,7 +7010,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Other open operation on femoral or popliteal artery OS</t>
+          <t>Diagnostic transluminal operation on other artery OS</t>
         </is>
       </c>
       <c r="H162" s="1" t="n">
@@ -7023,7 +7023,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>272129019</t>
+          <t>410979014</t>
         </is>
       </c>
       <c r="B163" s="1" t="n">
@@ -7031,12 +7031,12 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>7A5y</t>
+          <t>7A4A-3</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>7A5y.00</t>
+          <t>7A4A.13</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -7051,7 +7051,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Other specified operations on other artery</t>
+          <t>Other open operations on popliteal artery</t>
         </is>
       </c>
       <c r="H163" s="1" t="n">
@@ -7064,7 +7064,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>272104013</t>
+          <t>272129019</t>
         </is>
       </c>
       <c r="B164" s="1" t="n">
@@ -7072,12 +7072,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>7A53y</t>
+          <t>7A5y</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>7A53y00</t>
+          <t>7A5y.00</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Other specified other open operation on other artery</t>
+          <t>Other specified operations on other artery</t>
         </is>
       </c>
       <c r="H164" s="1" t="n">
@@ -9209,7 +9209,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>45851000006116</t>
+          <t>45861000006119</t>
         </is>
       </c>
       <c r="B217" s="1" t="n">
@@ -9217,12 +9217,12 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>7A23z</t>
+          <t>7A23y</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>7A23z00</t>
+          <t>7A23y00</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Operation on cerebral artery/ circle of Willis aneurysm NOS</t>
+          <t>Operation on cerebral artery/ circle of Willis aneurysm OS</t>
         </is>
       </c>
       <c r="H217" s="1" t="n">
@@ -9250,7 +9250,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>45861000006119</t>
+          <t>45851000006116</t>
         </is>
       </c>
       <c r="B218" s="1" t="n">
@@ -9258,12 +9258,12 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>7A23y</t>
+          <t>7A23z</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>7A23y00</t>
+          <t>7A23z00</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Operation on cerebral artery/ circle of Willis aneurysm OS</t>
+          <t>Operation on cerebral artery/ circle of Willis aneurysm NOS</t>
         </is>
       </c>
       <c r="H218" s="1" t="n">
@@ -9656,7 +9656,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>1587661000006116</t>
+          <t>1547961000006119</t>
         </is>
       </c>
       <c r="B228" s="1" t="n">
@@ -9664,12 +9664,12 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>7A0A6</t>
+          <t>7A0A4</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>7A0A600</t>
+          <t>7A0A400</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Percut transluminal balloon angioplasty pulmonary artery NEC</t>
+          <t>Percutaneous transluminal balloon angioplasty of pulmonary artery</t>
         </is>
       </c>
       <c r="H228" s="1" t="n">
@@ -9697,7 +9697,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>1547961000006119</t>
+          <t>1587661000006116</t>
         </is>
       </c>
       <c r="B229" s="1" t="n">
@@ -9705,12 +9705,12 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>7A0A4</t>
+          <t>7A0A6</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>7A0A400</t>
+          <t>7A0A600</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
@@ -9725,7 +9725,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Percutaneous transluminal balloon angioplasty of pulmonary artery</t>
+          <t>Percut transluminal balloon angioplasty pulmonary artery NEC</t>
         </is>
       </c>
       <c r="H229" s="1" t="n">
@@ -12060,7 +12060,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>271191011</t>
+          <t>271189015</t>
         </is>
       </c>
       <c r="B288" s="1" t="n">
@@ -12068,12 +12068,12 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>7932y</t>
+          <t>7932</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>7932y00</t>
+          <t>7932.00</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -12088,7 +12088,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Other specified open operation on heart</t>
+          <t>Other open operations on heart</t>
         </is>
       </c>
       <c r="H288" s="1" t="n">
@@ -12101,7 +12101,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>271189015</t>
+          <t>271191011</t>
         </is>
       </c>
       <c r="B289" s="1" t="n">
@@ -12109,12 +12109,12 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>7932</t>
+          <t>7932y</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>7932.00</t>
+          <t>7932y00</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Other open operations on heart</t>
+          <t>Other specified open operation on heart</t>
         </is>
       </c>
       <c r="H289" s="1" t="n">
@@ -12917,7 +12917,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>270854012</t>
+          <t>511571000000110</t>
         </is>
       </c>
       <c r="B309" s="1" t="n">
@@ -12925,12 +12925,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>790Az</t>
+          <t>7909-1</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>790Az00</t>
+          <t>7909.11</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -12945,20 +12945,20 @@
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>Other open operation on septum of heart NOS</t>
+          <t>Repair of defect of unspecified septum of heart</t>
         </is>
       </c>
       <c r="H309" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I309" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>270842012</t>
+          <t>270854012</t>
         </is>
       </c>
       <c r="B310" s="1" t="n">
@@ -12966,12 +12966,12 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>79092</t>
+          <t>790Az</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>7909200</t>
+          <t>790Az00</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -12986,20 +12986,20 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>Closure of defect of septum of heart using tissue graft NEC</t>
+          <t>Other open operation on septum of heart NOS</t>
         </is>
       </c>
       <c r="H310" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I310" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>511571000000110</t>
+          <t>270842012</t>
         </is>
       </c>
       <c r="B311" s="1" t="n">
@@ -13007,12 +13007,12 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>7909-1</t>
+          <t>79092</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>7909.11</t>
+          <t>7909200</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -13027,7 +13027,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Repair of defect of unspecified septum of heart</t>
+          <t>Closure of defect of septum of heart using tissue graft NEC</t>
         </is>
       </c>
       <c r="H311" s="1" t="n">
@@ -13360,7 +13360,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>271167019</t>
+          <t>271086012</t>
         </is>
       </c>
       <c r="B320" s="1" t="n">
@@ -13368,12 +13368,12 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>792Cy</t>
+          <t>7921z</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>792Cy00</t>
+          <t>7921z00</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -13388,7 +13388,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>Other specified replacement of coronary artery</t>
+          <t>Other autograft replacement of coronary artery NOS</t>
         </is>
       </c>
       <c r="H320" s="1" t="n">
@@ -13401,7 +13401,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>271086012</t>
+          <t>271167019</t>
         </is>
       </c>
       <c r="B321" s="1" t="n">
@@ -13409,12 +13409,12 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>7921z</t>
+          <t>792Cy</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>7921z00</t>
+          <t>792Cy00</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>Other autograft replacement of coronary artery NOS</t>
+          <t>Other specified replacement of coronary artery</t>
         </is>
       </c>
       <c r="H321" s="1" t="n">
@@ -14197,7 +14197,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>4312331000006112</t>
+          <t>272101017</t>
         </is>
       </c>
       <c r="B341" s="1" t="n">
@@ -14205,10 +14205,14 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>^ESCTPR431233</t>
-        </is>
-      </c>
-      <c r="D341" t="inlineStr"/>
+          <t>7A533</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>7A53300</t>
+        </is>
+      </c>
       <c r="E341" t="inlineStr">
         <is>
           <t>118805000</t>
@@ -14221,7 +14225,7 @@
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>Procedure on artery</t>
+          <t>Open cannulation of artery NEC</t>
         </is>
       </c>
       <c r="H341" s="1" t="n">
@@ -14234,7 +14238,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>272101017</t>
+          <t>4312331000006112</t>
         </is>
       </c>
       <c r="B342" s="1" t="n">
@@ -14242,14 +14246,10 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>7A533</t>
-        </is>
-      </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>7A53300</t>
-        </is>
-      </c>
+          <t>^ESCTPR431233</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
           <t>118805000</t>
@@ -14262,7 +14262,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Open cannulation of artery NEC</t>
+          <t>Procedure on artery</t>
         </is>
       </c>
       <c r="H342" s="1" t="n">
@@ -14755,7 +14755,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>807061000006110</t>
+          <t>271408019</t>
         </is>
       </c>
       <c r="B355" s="1" t="n">
@@ -14763,12 +14763,12 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>7A0y</t>
+          <t>7A0z</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>7A0y.00</t>
+          <t>7A0z.00</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>Great vessel or pulmonary artery operations OS</t>
+          <t>Great vessel and pulmonary artery operations NOS</t>
         </is>
       </c>
       <c r="H355" s="1" t="n">
@@ -14796,7 +14796,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>271408019</t>
+          <t>807061000006110</t>
         </is>
       </c>
       <c r="B356" s="1" t="n">
@@ -14804,12 +14804,12 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>7A0z</t>
+          <t>7A0y</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>7A0z.00</t>
+          <t>7A0y.00</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -14824,7 +14824,7 @@
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>Great vessel and pulmonary artery operations NOS</t>
+          <t>Great vessel or pulmonary artery operations OS</t>
         </is>
       </c>
       <c r="H356" s="1" t="n">
@@ -14997,7 +14997,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>270907012</t>
+          <t>271185014</t>
         </is>
       </c>
       <c r="B361" s="1" t="n">
@@ -15005,12 +15005,12 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>790H</t>
+          <t>79311</t>
         </is>
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>790H.00</t>
+          <t>7931100</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -15025,20 +15025,20 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>Other operations on wall of heart</t>
+          <t>Exploration of heart NEC</t>
         </is>
       </c>
       <c r="H361" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I361" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>271185014</t>
+          <t>451208015</t>
         </is>
       </c>
       <c r="B362" s="1" t="n">
@@ -15046,12 +15046,12 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>79311</t>
+          <t>790-4</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>7931100</t>
+          <t>790..14</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -15066,20 +15066,20 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>Exploration of heart NEC</t>
+          <t>Heart wall operations</t>
         </is>
       </c>
       <c r="H362" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I362" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>451208015</t>
+          <t>270907012</t>
         </is>
       </c>
       <c r="B363" s="1" t="n">
@@ -15087,12 +15087,12 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>790-4</t>
+          <t>790H</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>790..14</t>
+          <t>790H.00</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -15107,7 +15107,7 @@
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>Heart wall operations</t>
+          <t>Other operations on wall of heart</t>
         </is>
       </c>
       <c r="H363" s="1" t="n">
@@ -15481,7 +15481,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>270853018</t>
+          <t>14671000006119</t>
         </is>
       </c>
       <c r="B373" s="1" t="n">
@@ -15489,12 +15489,12 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>790Ay</t>
+          <t>7909y</t>
         </is>
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>790Ay00</t>
+          <t>7909y00</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -15509,20 +15509,20 @@
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>Other specified other open operation on septum of heart</t>
+          <t>Other specified closure of defect unspecified heart septum</t>
         </is>
       </c>
       <c r="H373" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I373" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>14671000006119</t>
+          <t>270853018</t>
         </is>
       </c>
       <c r="B374" s="1" t="n">
@@ -15530,12 +15530,12 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>7909y</t>
+          <t>790Ay</t>
         </is>
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>7909y00</t>
+          <t>790Ay00</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -15550,14 +15550,14 @@
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>Other specified closure of defect unspecified heart septum</t>
+          <t>Other specified other open operation on septum of heart</t>
         </is>
       </c>
       <c r="H374" s="1" t="n">
         <v>1</v>
       </c>
       <c r="I374" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="375">
@@ -15641,7 +15641,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>272105014</t>
+          <t>359411000000112</t>
         </is>
       </c>
       <c r="B377" s="1" t="n">
@@ -15649,12 +15649,12 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>7A53z</t>
+          <t>7A56</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>7A53z00</t>
+          <t>7A56.00</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -15669,7 +15669,7 @@
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>Other open operation on other artery NOS</t>
+          <t>Other therapeutic transluminal operations on artery</t>
         </is>
       </c>
       <c r="H377" s="1" t="n">
@@ -15682,7 +15682,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>359411000000112</t>
+          <t>105321000006118</t>
         </is>
       </c>
       <c r="B378" s="1" t="n">
@@ -15690,12 +15690,12 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>7A56</t>
+          <t>7A54y</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>7A56.00</t>
+          <t>7A54y00</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -15710,7 +15710,7 @@
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>Other therapeutic transluminal operations on artery</t>
+          <t>Therapeutic transluminal operation on other artery OS</t>
         </is>
       </c>
       <c r="H378" s="1" t="n">
@@ -15723,7 +15723,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>105321000006118</t>
+          <t>272105014</t>
         </is>
       </c>
       <c r="B379" s="1" t="n">
@@ -15731,12 +15731,12 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>7A54y</t>
+          <t>7A53z</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>7A54y00</t>
+          <t>7A53z00</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -15751,7 +15751,7 @@
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>Therapeutic transluminal operation on other artery OS</t>
+          <t>Other open operation on other artery NOS</t>
         </is>
       </c>
       <c r="H379" s="1" t="n">
@@ -15957,7 +15957,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>271406015</t>
+          <t>271405016</t>
         </is>
       </c>
       <c r="B385" s="1" t="n">
@@ -15965,12 +15965,12 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>7A0Az</t>
+          <t>7A0Ay</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>7A0Az00</t>
+          <t>7A0Ay00</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -15985,7 +15985,7 @@
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>Transluminal operation on pulmonary artery NOS</t>
+          <t>Other specified transluminal operation on pulmonary artery</t>
         </is>
       </c>
       <c r="H385" s="1" t="n">
@@ -15998,7 +15998,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>271405016</t>
+          <t>271406015</t>
         </is>
       </c>
       <c r="B386" s="1" t="n">
@@ -16006,12 +16006,12 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>7A0Ay</t>
+          <t>7A0Az</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>7A0Ay00</t>
+          <t>7A0Az00</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
@@ -16026,7 +16026,7 @@
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>Other specified transluminal operation on pulmonary artery</t>
+          <t>Transluminal operation on pulmonary artery NOS</t>
         </is>
       </c>
       <c r="H386" s="1" t="n">
@@ -16039,7 +16039,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>24131000006118</t>
+          <t>271544010</t>
         </is>
       </c>
       <c r="B387" s="1" t="n">
@@ -16047,12 +16047,12 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>7A24-1</t>
+          <t>7A21z</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>7A24.11</t>
+          <t>7A21z00</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -16067,7 +16067,7 @@
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>Other open operations on cerebral artery</t>
+          <t>Other open operation on carotid artery NOS</t>
         </is>
       </c>
       <c r="H387" s="1" t="n">
@@ -16080,7 +16080,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>271544010</t>
+          <t>271543016</t>
         </is>
       </c>
       <c r="B388" s="1" t="n">
@@ -16088,12 +16088,12 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>7A21z</t>
+          <t>7A21y</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>7A21z00</t>
+          <t>7A21y00</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -16108,7 +16108,7 @@
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>Other open operation on carotid artery NOS</t>
+          <t>Other specified other open operation on carotid artery</t>
         </is>
       </c>
       <c r="H388" s="1" t="n">
@@ -16121,7 +16121,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>271644017</t>
+          <t>24131000006118</t>
         </is>
       </c>
       <c r="B389" s="1" t="n">
@@ -16129,12 +16129,12 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>7A27y</t>
+          <t>7A24-1</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>7A27y00</t>
+          <t>7A24.11</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>Other specified other open operation on subclavian artery</t>
+          <t>Other open operations on cerebral artery</t>
         </is>
       </c>
       <c r="H389" s="1" t="n">
@@ -16162,7 +16162,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>271543016</t>
+          <t>271645016</t>
         </is>
       </c>
       <c r="B390" s="1" t="n">
@@ -16170,12 +16170,12 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>7A21y</t>
+          <t>7A27z</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>7A21y00</t>
+          <t>7A27z00</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
@@ -16190,7 +16190,7 @@
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>Other specified other open operation on carotid artery</t>
+          <t>Other open operation on subclavian artery NOS</t>
         </is>
       </c>
       <c r="H390" s="1" t="n">
@@ -16203,7 +16203,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>271645016</t>
+          <t>271644017</t>
         </is>
       </c>
       <c r="B391" s="1" t="n">
@@ -16211,12 +16211,12 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>7A27z</t>
+          <t>7A27y</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>7A27z00</t>
+          <t>7A27y00</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -16231,7 +16231,7 @@
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>Other open operation on subclavian artery NOS</t>
+          <t>Other specified other open operation on subclavian artery</t>
         </is>
       </c>
       <c r="H391" s="1" t="n">
@@ -16244,7 +16244,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>271550017</t>
+          <t>271551018</t>
         </is>
       </c>
       <c r="B392" s="1" t="n">
@@ -16252,12 +16252,12 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>7A22y</t>
+          <t>7A22z</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>7A22y00</t>
+          <t>7A22z00</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>Other specified transluminal operation on carotid artery</t>
+          <t>Transluminal operation on carotid artery NOS</t>
         </is>
       </c>
       <c r="H392" s="1" t="n">
@@ -16285,7 +16285,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>271551018</t>
+          <t>271550017</t>
         </is>
       </c>
       <c r="B393" s="1" t="n">
@@ -16293,12 +16293,12 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>7A22z</t>
+          <t>7A22y</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>7A22z00</t>
+          <t>7A22y00</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t>Transluminal operation on carotid artery NOS</t>
+          <t>Other specified transluminal operation on carotid artery</t>
         </is>
       </c>
       <c r="H393" s="1" t="n">
@@ -16367,7 +16367,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>349457013</t>
+          <t>349459011</t>
         </is>
       </c>
       <c r="B395" s="1" t="n">
@@ -16375,12 +16375,12 @@
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>7A34-3</t>
+          <t>7A34-1</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>7A34.13</t>
+          <t>7A34.11</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -16395,7 +16395,7 @@
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t>Other open operations on superior mesenteric artery</t>
+          <t>Other open operations on coeliac artery</t>
         </is>
       </c>
       <c r="H395" s="1" t="n">
@@ -16408,7 +16408,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>349458015</t>
+          <t>349457013</t>
         </is>
       </c>
       <c r="B396" s="1" t="n">
@@ -16416,12 +16416,12 @@
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>7A34-2</t>
+          <t>7A34-3</t>
         </is>
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>7A34.12</t>
+          <t>7A34.13</t>
         </is>
       </c>
       <c r="E396" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>Other open operations on inferior mesenteric artery</t>
+          <t>Other open operations on superior mesenteric artery</t>
         </is>
       </c>
       <c r="H396" s="1" t="n">
@@ -16449,7 +16449,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>349459011</t>
+          <t>349458015</t>
         </is>
       </c>
       <c r="B397" s="1" t="n">
@@ -16457,12 +16457,12 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>7A34-1</t>
+          <t>7A34-2</t>
         </is>
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>7A34.11</t>
+          <t>7A34.12</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -16477,7 +16477,7 @@
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t>Other open operations on coeliac artery</t>
+          <t>Other open operations on inferior mesenteric artery</t>
         </is>
       </c>
       <c r="H397" s="1" t="n">
@@ -16925,7 +16925,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>394315016</t>
+          <t>271676010</t>
         </is>
       </c>
       <c r="B409" s="1" t="n">
@@ -16933,12 +16933,12 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>7A28</t>
+          <t>7A28y</t>
         </is>
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>7A28.00</t>
+          <t>7A28y00</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -16953,7 +16953,7 @@
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t>Transluminal operations on subclavian artery</t>
+          <t>Other specified transluminal operation on subclavian artery</t>
         </is>
       </c>
       <c r="H409" s="1" t="n">
@@ -16966,7 +16966,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>271676010</t>
+          <t>394315016</t>
         </is>
       </c>
       <c r="B410" s="1" t="n">
@@ -16974,12 +16974,12 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>7A28y</t>
+          <t>7A28</t>
         </is>
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>7A28y00</t>
+          <t>7A28.00</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="G410" t="inlineStr">
         <is>
-          <t>Other specified transluminal operation on subclavian artery</t>
+          <t>Transluminal operations on subclavian artery</t>
         </is>
       </c>
       <c r="H410" s="1" t="n">
@@ -18681,7 +18681,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>356421000000114</t>
+          <t>376941000000111</t>
         </is>
       </c>
       <c r="B453" s="1" t="n">
@@ -18689,12 +18689,12 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>793H</t>
+          <t>793Hy</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>793H.00</t>
+          <t>793Hy00</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
@@ -18709,7 +18709,7 @@
       </c>
       <c r="G453" t="inlineStr">
         <is>
-          <t>Transluminal operations on cardiac conduit</t>
+          <t>Other specified transluminal operations on cardiac conduit</t>
         </is>
       </c>
       <c r="H453" s="1" t="n">
@@ -18722,7 +18722,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>376941000000111</t>
+          <t>356421000000114</t>
         </is>
       </c>
       <c r="B454" s="1" t="n">
@@ -18730,12 +18730,12 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>793Hy</t>
+          <t>793H</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>793Hy00</t>
+          <t>793H.00</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
@@ -18750,7 +18750,7 @@
       </c>
       <c r="G454" t="inlineStr">
         <is>
-          <t>Other specified transluminal operations on cardiac conduit</t>
+          <t>Transluminal operations on cardiac conduit</t>
         </is>
       </c>
       <c r="H454" s="1" t="n">
@@ -21649,7 +21649,7 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>271775016</t>
+          <t>271779010</t>
         </is>
       </c>
       <c r="B529" s="1" t="n">
@@ -21657,12 +21657,12 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>7A34C</t>
+          <t>7A34F</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>7A34C00</t>
+          <t>7A34F00</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
@@ -21677,7 +21677,7 @@
       </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>Operation on aneurysm of coeliac artery NEC</t>
+          <t>Operation on aneurysm of suprarenal artery NEC</t>
         </is>
       </c>
       <c r="H529" s="1" t="n">
@@ -21690,7 +21690,7 @@
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>271779010</t>
+          <t>271775016</t>
         </is>
       </c>
       <c r="B530" s="1" t="n">
@@ -21698,12 +21698,12 @@
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>7A34F</t>
+          <t>7A34C</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>7A34F00</t>
+          <t>7A34C00</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
@@ -21718,7 +21718,7 @@
       </c>
       <c r="G530" t="inlineStr">
         <is>
-          <t>Operation on aneurysm of suprarenal artery NEC</t>
+          <t>Operation on aneurysm of coeliac artery NEC</t>
         </is>
       </c>
       <c r="H530" s="1" t="n">
@@ -27108,7 +27108,7 @@
     <row r="672">
       <c r="A672" t="inlineStr">
         <is>
-          <t>187951000006118</t>
+          <t>271744013</t>
         </is>
       </c>
       <c r="B672" s="1" t="n">
@@ -27116,12 +27116,12 @@
       </c>
       <c r="C672" t="inlineStr">
         <is>
-          <t>7A33y</t>
+          <t>7A33J</t>
         </is>
       </c>
       <c r="D672" t="inlineStr">
         <is>
-          <t>7A33y00</t>
+          <t>7A33J00</t>
         </is>
       </c>
       <c r="E672" t="inlineStr">
@@ -27136,7 +27136,7 @@
       </c>
       <c r="G672" t="inlineStr">
         <is>
-          <t>Reconstruction of other visceral branch abdominal aorta OS</t>
+          <t>Replantation of visceral branch of abdominal aorta NEC</t>
         </is>
       </c>
       <c r="H672" s="1" t="n">
@@ -27149,7 +27149,7 @@
     <row r="673">
       <c r="A673" t="inlineStr">
         <is>
-          <t>271726017</t>
+          <t>271730019</t>
         </is>
       </c>
       <c r="B673" s="1" t="n">
@@ -27157,12 +27157,12 @@
       </c>
       <c r="C673" t="inlineStr">
         <is>
-          <t>7A334</t>
+          <t>7A337</t>
         </is>
       </c>
       <c r="D673" t="inlineStr">
         <is>
-          <t>7A33400</t>
+          <t>7A33700</t>
         </is>
       </c>
       <c r="E673" t="inlineStr">
@@ -27177,7 +27177,7 @@
       </c>
       <c r="G673" t="inlineStr">
         <is>
-          <t>Replantation of coeliac artery NEC</t>
+          <t>Replantation of suprarenal artery NEC</t>
         </is>
       </c>
       <c r="H673" s="1" t="n">
@@ -27190,7 +27190,7 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>271730019</t>
+          <t>187951000006118</t>
         </is>
       </c>
       <c r="B674" s="1" t="n">
@@ -27198,12 +27198,12 @@
       </c>
       <c r="C674" t="inlineStr">
         <is>
-          <t>7A337</t>
+          <t>7A33y</t>
         </is>
       </c>
       <c r="D674" t="inlineStr">
         <is>
-          <t>7A33700</t>
+          <t>7A33y00</t>
         </is>
       </c>
       <c r="E674" t="inlineStr">
@@ -27218,7 +27218,7 @@
       </c>
       <c r="G674" t="inlineStr">
         <is>
-          <t>Replantation of suprarenal artery NEC</t>
+          <t>Reconstruction of other visceral branch abdominal aorta OS</t>
         </is>
       </c>
       <c r="H674" s="1" t="n">
@@ -27231,7 +27231,7 @@
     <row r="675">
       <c r="A675" t="inlineStr">
         <is>
-          <t>271744013</t>
+          <t>271726017</t>
         </is>
       </c>
       <c r="B675" s="1" t="n">
@@ -27239,12 +27239,12 @@
       </c>
       <c r="C675" t="inlineStr">
         <is>
-          <t>7A33J</t>
+          <t>7A334</t>
         </is>
       </c>
       <c r="D675" t="inlineStr">
         <is>
-          <t>7A33J00</t>
+          <t>7A33400</t>
         </is>
       </c>
       <c r="E675" t="inlineStr">
@@ -27259,7 +27259,7 @@
       </c>
       <c r="G675" t="inlineStr">
         <is>
-          <t>Replantation of visceral branch of abdominal aorta NEC</t>
+          <t>Replantation of coeliac artery NEC</t>
         </is>
       </c>
       <c r="H675" s="1" t="n">

</xml_diff>